<commit_message>
Update example test file DefiningRanges
Update reference test file for example DefiningRanges. After
style infrastructure switch, the styles part is saved differently.
The test file has been updated, no semantic change.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Ranges/DefiningRanges.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Ranges/DefiningRanges.xlsx
@@ -31,61 +31,52 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>